<commit_message>
refactor: update agent workflows and skills for individual equity cards
- Split bulk equity files into individual markdown cards
- Update all automation scripts for the new data structure
- Refactor web dashboard to fetch data from GitHub API
- Add data quality checks for Country/Territory fields
- Fix dashboard repo slug and button logic
- Update documentation and workflows
</commit_message>
<xml_diff>
--- a/published/02_Grants_Active.xlsx
+++ b/published/02_Grants_Active.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Active_Grants" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Active_Grants" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Active_Grants'!$A$1:$H$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Active_Grants'!$A$1:$H$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,16 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,19 +60,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -444,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -505,37 +496,37 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Grants for Developing Internationalisation Strategies for SMEs (Malta)</t>
+          <t>Grant Opportunity: CABHI’s Fuel Program in Canada</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>The Internationalisation Strategy for SMEs scheme helps SMEs access expert support in developing strategies to improve efficiency, competitiveness, and international market readiness. The scheme supports studying opportunities abroad and developing strategies for selected countries, including marketing and sales plans and risk assessment.</t>
+          <t>The Centre for Aging + Brain Health Innovation is accepting applications for its Fuel program, designed to remove barriers and accelerate innovative solutions that have the potential to transform the aging experience. The program supports start-up companies and healthcare/research organizations in advancing innovations and achieving validation milestones.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>FONDI.eu (Government of Malta)</t>
+          <t>CABHI (Centre for Aging + Brain Health Innovation)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Maximum €20,000 per undertaking</t>
+          <t>Up to $500,000 CAD</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>International market readiness, market feasibility, entry strategy, smart economic transformation</t>
+          <t>Aging, Brain Health, Healthcare Innovation</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>https://fondi.eu/what-funding-is-available/internationalisation-strategy-for-smes/</t>
+          <t>https://www.cabhi.com/en/innovation-programs-services/fuel</t>
         </is>
       </c>
     </row>
@@ -545,37 +536,37 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Grant Opportunity: CFAs: Standards and Awards Support for SMEs (Malta)</t>
+          <t>Grant Opportunity: Funding for Consolidated Research Infrastructure Clusters</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The Standards &amp; Awards for SMEs scheme assists small and medium-sized enterprises in strengthening their business operations and attaining prestigious national or international standards and awards. The scheme focuses on enhancing competitiveness and credibility through internationally recognized certifications or national excellence awards.</t>
+          <t>The European Commission is advancing efforts to strengthen and streamline its research infrastructure ecosystem by supporting initiatives that improve coordination, accessibility, and policy engagement across large thematic domains. The programme aims to equip large thematic clusters of European research infrastructures with both a policy-oriented and a technical framework to better represent their collective interests and enhance collaboration across the research ecosystem.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>FONDI.eu (Government of Malta)</t>
+          <t>European Commission</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Maximum €15,000 (up to €20,000 for multiple standards)</t>
+          <t>€4,000,000 to €8,000,000 per project (Total budget: €40,000,000)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Internationally recognized certifications, national excellence awards, quality, efficiency, sustainability</t>
+          <t>Research Infrastructure, Policy Engagement, Technological Framework, Innovation</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://fondi.eu/what-funding-is-available/standards-awards-for-smes/</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-INFRA-2026-DEV-01-02?order=DESC&amp;pageNumber=1&amp;pageSize=50&amp;sortBy=startDate&amp;isExactMatch=true&amp;status=31094502</t>
         </is>
       </c>
     </row>
@@ -585,37 +576,37 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Funding for Consolidated Research Infrastructure Clusters</t>
+          <t>Grant Opportunity: Open Call: Marketing Strategy Support Grant for SMEs (Malta)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>The European Commission is advancing efforts to strengthen and streamline its research infrastructure ecosystem by supporting initiatives that improve coordination, accessibility, and policy engagement across large thematic domains. The programme aims to equip large thematic clusters of European research infrastructures with both a policy-oriented and a technical framework to better represent their collective interests and enhance collaboration across the research ecosystem.</t>
+          <t>The Marketing Strategy for Micro &amp; Small Enterprises scheme supports micro and small businesses in obtaining professional guidance to design marketing strategies that boost their competitiveness and drive business growth. It part-finances costs incurred for external services contracted to deliver a marketing strategy aligned with the enterprise’s objectives.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>European Commission</t>
+          <t>FONDI.eu (Government of Malta)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>€4,000,000 to €8,000,000 per project (Total budget: €40,000,000)</t>
+          <t>Maximum €10,000</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Research Infrastructure, Policy Engagement, Technological Framework, Innovation</t>
+          <t>Marketing strategy, business promotion, competitiveness, smart economic transformation</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-INFRA-2026-DEV-01-02?order=DESC&amp;pageNumber=1&amp;pageSize=50&amp;sortBy=startDate&amp;isExactMatch=true&amp;status=31094502</t>
+          <t>https://fondi.eu/what-funding-is-available/marketing-strategy-for-smes/</t>
         </is>
       </c>
     </row>
@@ -625,37 +616,37 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Applications open for Private Sector Pathways Program (Australia)</t>
+          <t>Grant Opportunity: Grants for Developing Internationalisation Strategies for SMEs (Malta)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>The Private Sector Pathways Program is inviting applications to support innovative small-to-medium enterprises in Queensland to collaborate with corporate partners and develop commercialisation opportunities. The program focuses on increasing partnerships between SMEs and corporate businesses or large organisations to solve problems and trial technologies.</t>
+          <t>The Internationalisation Strategy for SMEs scheme helps SMEs access expert support in developing strategies to improve efficiency, competitiveness, and international market readiness. The scheme supports studying opportunities abroad and developing strategies for selected countries, including marketing and sales plans and risk assessment.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Australian Government (Queensland)</t>
+          <t>FONDI.eu (Government of Malta)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-04-14</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Up to $100,000</t>
+          <t>Maximum €20,000 per undertaking</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Commercialisation opportunities, SME-Corporate partnerships, advanced manufacturing, hydrogen, biomedical, aerospace</t>
+          <t>International market readiness, market feasibility, entry strategy, smart economic transformation</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://business.gov.au/grants-and-programs/private-sector-pathways-program-qld</t>
+          <t>https://fondi.eu/what-funding-is-available/internationalisation-strategy-for-smes/</t>
         </is>
       </c>
     </row>
@@ -665,37 +656,37 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Entries Open for Cyber Valley AI Incubator Program</t>
+          <t>Grant Opportunity: Take Your Shot Program Entrepreneurship Program (Canada)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>The Cyber Valley AI Incubator offers a practical platform for researchers, technologists, and innovators to develop and launch AI-driven ventures. The program provides a collaborative environment where participants can develop their ideas into tangible ventures, leveraging world-class research and expertise.</t>
+          <t>The Take Your Shot program is an entrepreneurship program inviting applications from young entrepreneurs to develop their business ideas with funding and professional mentorship. The program includes mandatory workshops and a final pitch event where participants can present their ideas to a panel of judges.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Cyber Valley</t>
+          <t>The Bridge Youth Resource Centre</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not specified (Incubator program with practical platform and expertise)</t>
+          <t>Up to $20,000 (Scholarship/Awards)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Artificial Intelligence, Machine Learning, Robotics, Intelligent Systems, Data Science, Biomedical Technology</t>
+          <t>Entrepreneurship, mentorship, workshops, marketing, branding, financial planning</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>https://ai-incubator.is.mpg.de/</t>
+          <t>https://thebridgeyouth.ca/take-your-shot/</t>
         </is>
       </c>
     </row>
@@ -705,37 +696,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Open Call for Low Emissions Industry Program in Australia</t>
+          <t>Grant Opportunity: Funding Call for Space-Tech Wetland Sustainability Projects</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>The Low Emissions Industry Program supports projects that reduce emissions in mining and manufacturing facilities while strengthening their transition toward a low-carbon future. The program focuses on driving emissions reductions by co-funding projects, future-proofing industrial assets, and maintaining economic resilience.</t>
+          <t>The European Space Agency is seeking applications to develop space-enabled applications that support wetland sustainability and create viable business opportunities. The opportunity supports feasibility studies over a six-month period for early-stage service concepts that respond to real customer needs while demonstrating technical feasibility and commercial potential.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Australian Government (Department of Climate Change, Energy, the Environment and Water)</t>
+          <t>European Space Agency (ESA)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>$500,000 to $10 million</t>
+          <t>Up to €75,000 per activity (75% of total project cost)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Emissions reduction in mining and manufacturing, transition to net zero</t>
+          <t>Space-enabled applications for wetland sustainability, water purification, flood control, biodiversity support</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://business.gov.au/grants-and-programs/low-emissions-industry-program-nsw</t>
+          <t>https://business.esa.int/funding/call-for-proposals-competitive/sustainable-wetlands</t>
         </is>
       </c>
     </row>
@@ -745,37 +736,37 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Waste Minimisation Fund in New Zealand</t>
+          <t>Grant Opportunity: Funding to Support SMEs’ Business Reports and Plans (Malta)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>The Waste Minimisation Fund is seeking applications to support innovative projects that reduce waste, improve resource efficiency, and encourage community participation, education, and long-term behaviour change across the Whangārei District. The fund focuses on complementing and enhancing existing waste minimisation programmes and creating new opportunities for reducing waste.</t>
+          <t>The Business Reports for SMEs Grant Scheme offers funding to support SMEs in creating external consultancy reports to improve efficiency, competitiveness, and investment readiness. It provides financial support to contract external expertise needed to generate high-quality business reports that inform strategic decisions and strengthen operational performance.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Whangārei District Council</t>
+          <t>FONDI.eu (Government of Malta)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Standard grants ranging from $1,000 to $5,000 and special project grants from $5,000 to $30,000</t>
+          <t>Lump sum of €4,000 (80% aid intensity)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Waste Minimisation, Resource Efficiency, Community Participation</t>
+          <t>External consultancy reports, efficiency, competitiveness, investment readiness</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>https://www.wdc.govt.nz/Community/Community-funding/Waste-Minimisation-Fund</t>
+          <t>https://fondi.eu/what-funding-is-available/business-reports-for-smes/</t>
         </is>
       </c>
     </row>
@@ -785,37 +776,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Advancing Digital Twins for Climate, Environment and Security</t>
+          <t>Grant Opportunity: Waste Minimisation Fund in New Zealand</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>The European Commission is supporting initiatives to develop advanced digital twin technologies that strengthen preparedness, resilience and decision-making in response to the growing security challenges linked to climate and environmental change. The initiative focuses on improving security and preparedness for the Union and creating a more disaster-resilient society in the face of climate change impacts.</t>
+          <t>The Waste Minimisation Fund is seeking applications to support innovative projects that reduce waste, improve resource efficiency, and encourage community participation, education, and long-term behaviour change across the Whangārei District. The fund focuses on complementing and enhancing existing waste minimisation programmes and creating new opportunities for reducing waste.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>European Commission</t>
+          <t>Whangārei District Council</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>€5,000,000 to €7,500,000 per project (Total budget: €15,000,000)</t>
+          <t>Standard grants ranging from $1,000 to $5,000 and special project grants from $5,000 to $30,000</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Digital Twins, Climate Change, Environment, Security, AI</t>
+          <t>Waste Minimisation, Resource Efficiency, Community Participation</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-INFRA-2026-TECH-01-02?order=DESC&amp;pageNumber=1&amp;pageSize=50&amp;sortBy=startDate&amp;isExactMatch=true&amp;status=31094502</t>
+          <t>https://www.wdc.govt.nz/Community/Community-funding/Waste-Minimisation-Fund</t>
         </is>
       </c>
     </row>
@@ -825,37 +816,37 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Take Your Shot Program Entrepreneurship Program (Canada)</t>
+          <t>Grant Opportunity: CFAs: Standards and Awards Support for SMEs (Malta)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>The Take Your Shot program is an entrepreneurship program inviting applications from young entrepreneurs to develop their business ideas with funding and professional mentorship. The program includes mandatory workshops and a final pitch event where participants can present their ideas to a panel of judges.</t>
+          <t>The Standards &amp; Awards for SMEs scheme assists small and medium-sized enterprises in strengthening their business operations and attaining prestigious national or international standards and awards. The scheme focuses on enhancing competitiveness and credibility through internationally recognized certifications or national excellence awards.</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>The Bridge Youth Resource Centre</t>
+          <t>FONDI.eu (Government of Malta)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-17</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Up to $20,000 (Scholarship/Awards)</t>
+          <t>Maximum €15,000 (up to €20,000 for multiple standards)</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Entrepreneurship, mentorship, workshops, marketing, branding, financial planning</t>
+          <t>Internationally recognized certifications, national excellence awards, quality, efficiency, sustainability</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>https://thebridgeyouth.ca/take-your-shot/</t>
+          <t>https://fondi.eu/what-funding-is-available/standards-awards-for-smes/</t>
         </is>
       </c>
     </row>
@@ -865,17 +856,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Grant Opportunity: CABHI’s Fuel Program in Canada</t>
+          <t>Grant Opportunity: Entries Open for Cyber Valley AI Incubator Program</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>The Centre for Aging + Brain Health Innovation is accepting applications for its Fuel program, designed to remove barriers and accelerate innovative solutions that have the potential to transform the aging experience. The program supports start-up companies and healthcare/research organizations in advancing innovations and achieving validation milestones.</t>
+          <t>The Cyber Valley AI Incubator offers a practical platform for researchers, technologists, and innovators to develop and launch AI-driven ventures. The program provides a collaborative environment where participants can develop their ideas into tangible ventures, leveraging world-class research and expertise.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>CABHI (Centre for Aging + Brain Health Innovation)</t>
+          <t>Cyber Valley</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -885,17 +876,17 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Up to $500,000 CAD</t>
+          <t>Not specified (Incubator program with practical platform and expertise)</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Aging, Brain Health, Healthcare Innovation</t>
+          <t>Artificial Intelligence, Machine Learning, Robotics, Intelligent Systems, Data Science, Biomedical Technology</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://www.cabhi.com/en/innovation-programs-services/fuel</t>
+          <t>https://ai-incubator.is.mpg.de/</t>
         </is>
       </c>
     </row>
@@ -905,37 +896,37 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Funding to Support SMEs’ Business Reports and Plans (Malta)</t>
+          <t>Grant Opportunity: Open Call for Low Emissions Industry Program in Australia</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>The Business Reports for SMEs Grant Scheme offers funding to support SMEs in creating external consultancy reports to improve efficiency, competitiveness, and investment readiness. It provides financial support to contract external expertise needed to generate high-quality business reports that inform strategic decisions and strengthen operational performance.</t>
+          <t>The Low Emissions Industry Program supports projects that reduce emissions in mining and manufacturing facilities while strengthening their transition toward a low-carbon future. The program focuses on driving emissions reductions by co-funding projects, future-proofing industrial assets, and maintaining economic resilience.</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>FONDI.eu (Government of Malta)</t>
+          <t>Australian Government (Department of Climate Change, Energy, the Environment and Water)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Lump sum of €4,000 (80% aid intensity)</t>
+          <t>$500,000 to $10 million</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>External consultancy reports, efficiency, competitiveness, investment readiness</t>
+          <t>Emissions reduction in mining and manufacturing, transition to net zero</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>https://fondi.eu/what-funding-is-available/business-reports-for-smes/</t>
+          <t>https://business.gov.au/grants-and-programs/low-emissions-industry-program-nsw</t>
         </is>
       </c>
     </row>
@@ -945,82 +936,42 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Grant Opportunity: Open Call: Marketing Strategy Support Grant for SMEs (Malta)</t>
+          <t>Grant Opportunity: Advancing Digital Twins for Climate, Environment and Security</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>The Marketing Strategy for Micro &amp; Small Enterprises scheme supports micro and small businesses in obtaining professional guidance to design marketing strategies that boost their competitiveness and drive business growth. It part-finances costs incurred for external services contracted to deliver a marketing strategy aligned with the enterprise’s objectives.</t>
+          <t>The European Commission is supporting initiatives to develop advanced digital twin technologies that strengthen preparedness, resilience and decision-making in response to the growing security challenges linked to climate and environmental change. The initiative focuses on improving security and preparedness for the Union and creating a more disaster-resilient society in the face of climate change impacts.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>FONDI.eu (Government of Malta)</t>
+          <t>European Commission</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2026-04-17</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Maximum €10,000</t>
+          <t>€5,000,000 to €7,500,000 per project (Total budget: €15,000,000)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Marketing strategy, business promotion, competitiveness, smart economic transformation</t>
+          <t>Digital Twins, Climate Change, Environment, Security, AI</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://fondi.eu/what-funding-is-available/marketing-strategy-for-smes/</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Grant Opportunity: Funding Call for Space-Tech Wetland Sustainability Projects</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>The European Space Agency is seeking applications to develop space-enabled applications that support wetland sustainability and create viable business opportunities. The opportunity supports feasibility studies over a six-month period for early-stage service concepts that respond to real customer needs while demonstrating technical feasibility and commercial potential.</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>European Space Agency (ESA)</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-15</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Up to €75,000 per activity (75% of total project cost)</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Space-enabled applications for wetland sustainability, water purification, flood control, biodiversity support</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>https://business.esa.int/funding/call-for-proposals-competitive/sustainable-wetlands</t>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/topic-details/HORIZON-INFRA-2026-TECH-01-02?order=DESC&amp;pageNumber=1&amp;pageSize=50&amp;sortBy=startDate&amp;isExactMatch=true&amp;status=31094502</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>